<commit_message>
Gestion dynamique des fiches techniques avec recalcul en direct du Food Cost, sauvegarde persistante et synchronisation
</commit_message>
<xml_diff>
--- a/prix d'achats des produits.xlsx
+++ b/prix d'achats des produits.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3289701b0f721e94/Dokumente/GitHub/Fiche-technique/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{95C24205-5325-4BB4-883C-5A63AF7D7997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{95C24205-5325-4BB4-883C-5A63AF7D7997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A99DD99-85B4-480D-945D-3CF6CF9CC4E8}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D1880E55-4320-4990-978F-5D008D1EE88A}"/>
   </bookViews>
@@ -2536,7 +2536,7 @@
         <v>101</v>
       </c>
       <c r="B87" s="5">
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="C87" s="5" t="s">
         <v>9</v>

</xml_diff>